<commit_message>
used pivot table for the whole data for region and its cost
</commit_message>
<xml_diff>
--- a/EXCEL/Interactive Chart Dropdown.xlsx
+++ b/EXCEL/Interactive Chart Dropdown.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{CDCD8BA8-1731-43EF-A390-AA5DE34312B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF2D42DE-BBF0-4036-A496-785535F24FBF}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{CDCD8BA8-1731-43EF-A390-AA5DE34312B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{102390A5-76DF-4BF1-9D60-157BEE3241CD}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{45E58E42-5660-421A-ADBC-2E6097C92F70}"/>
+    <workbookView minimized="1" xWindow="2112" yWindow="1836" windowWidth="17280" windowHeight="10428" xr2:uid="{45E58E42-5660-421A-ADBC-2E6097C92F70}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="21">
   <si>
     <t>Month</t>
   </si>
@@ -108,6 +108,24 @@
   </si>
   <si>
     <t>Region wise Data</t>
+  </si>
+  <si>
+    <t>Product A</t>
+  </si>
+  <si>
+    <t>Product B</t>
+  </si>
+  <si>
+    <t>Product C</t>
+  </si>
+  <si>
+    <t>Leads</t>
+  </si>
+  <si>
+    <t>Qualified</t>
+  </si>
+  <si>
+    <t>Converted</t>
   </si>
 </sst>
 </file>
@@ -139,7 +157,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -147,11 +165,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -161,6 +194,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1504,7 +1546,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0403E043-6B0F-4163-812F-9898E4866638}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:9" ht="42" x14ac:dyDescent="0.4">
@@ -1674,6 +1716,99 @@
       </c>
       <c r="D9" s="2">
         <v>1500</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45"/>
+    <row r="16" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" s="6">
+        <v>3000</v>
+      </c>
+      <c r="C17" s="6">
+        <v>2000</v>
+      </c>
+      <c r="D17" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E17" s="6">
+        <v>500</v>
+      </c>
+      <c r="F17" s="6">
+        <v>300</v>
+      </c>
+      <c r="G17" s="6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="6">
+        <v>3500</v>
+      </c>
+      <c r="C18" s="6">
+        <v>2500</v>
+      </c>
+      <c r="D18" s="6">
+        <v>1500</v>
+      </c>
+      <c r="E18" s="6">
+        <v>600</v>
+      </c>
+      <c r="F18" s="6">
+        <v>350</v>
+      </c>
+      <c r="G18" s="6">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="6">
+        <v>4000</v>
+      </c>
+      <c r="C19" s="6">
+        <v>3000</v>
+      </c>
+      <c r="D19" s="6">
+        <v>2000</v>
+      </c>
+      <c r="E19" s="6">
+        <v>700</v>
+      </c>
+      <c r="F19" s="6">
+        <v>400</v>
+      </c>
+      <c r="G19" s="6">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>